<commit_message>
Update rosters with jersey numbers, positions, and grad years; Steilacoom DH times
- Roster: added Positions and Grad Year columns with actual jersey numbers from spreadsheet
- Roster: name fixes (Greyson Riley, Jonah Vitcovich, Gabe LaPlante)
- CSS: fix responsive rule hiding Grad Year header on roster page
- CSS: widen roster table for new columns, bump cache version to v=5
- C Team Steilacoom DH: set game times to 12:00 PM & 2:00 PM
- C Team stats: 58 total events (split Steilacoom into G1/G2)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schedule/2026 Master Schedule.xlsx
+++ b/Schedule/2026 Master Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bsleeter/Documents/Documents - Benjamin's MacBook Pro/GH Baseball/Schedule/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C38F81F7-A40D-424C-A7B0-2F8E4EDF12FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2416402E-9D59-3044-8065-8BE5B11F26C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="160" yWindow="1140" windowWidth="27300" windowHeight="16500" activeTab="1" xr2:uid="{DEE07C68-23DA-2F4F-8E1C-1A71F8558C8E}"/>
   </bookViews>
@@ -669,9 +669,6 @@
     <t>Game vs Seillacoom (DH)</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t xml:space="preserve">Game vs PHS </t>
   </si>
   <si>
@@ -739,6 +736,9 @@
   </si>
   <si>
     <t>8:00am - 3:00 pm</t>
+  </si>
+  <si>
+    <t>12pm, 2pm</t>
   </si>
 </sst>
 </file>
@@ -2734,7 +2734,7 @@
         <v>147</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>142</v>
@@ -2787,7 +2787,7 @@
         <v>146</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>5</v>
@@ -2809,7 +2809,7 @@
         <v>14</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -2862,7 +2862,7 @@
         <v>148</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>151</v>
@@ -2904,7 +2904,7 @@
         <v>149</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>151</v>
@@ -2977,7 +2977,7 @@
         <v>14</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
@@ -2988,7 +2988,7 @@
         <v>150</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>142</v>
@@ -2997,7 +2997,7 @@
         <v>150</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>185</v>
@@ -3006,10 +3006,10 @@
         <v>201</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>18</v>
@@ -3088,7 +3088,7 @@
         <v>154</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>156</v>
@@ -3097,7 +3097,7 @@
         <v>189</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>156</v>
@@ -3148,7 +3148,7 @@
         <v>146</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J19" s="11" t="s">
         <v>5</v>
@@ -3232,7 +3232,7 @@
         <v>146</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J21" s="11" t="s">
         <v>5</v>
@@ -3311,7 +3311,7 @@
         <v>146</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G24" s="8" t="s">
         <v>5</v>
@@ -3353,7 +3353,7 @@
         <v>191</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G25" s="8" t="s">
         <v>160</v>
@@ -3404,7 +3404,7 @@
         <v>146</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="J26" s="11" t="s">
         <v>5</v>
@@ -3512,7 +3512,7 @@
         <v>161</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>142</v>
@@ -3524,7 +3524,7 @@
         <v>209</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>210</v>
+        <v>233</v>
       </c>
       <c r="J29" s="11" t="s">
         <v>185</v>
@@ -3571,7 +3571,7 @@
         <v>146</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G31" s="8" t="s">
         <v>186</v>
@@ -3619,7 +3619,7 @@
         <v>165</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="I32" s="11" t="s">
         <v>202</v>
@@ -3646,7 +3646,7 @@
         <v>164</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>165</v>
@@ -3739,7 +3739,7 @@
         <v>146</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G35" s="8" t="s">
         <v>186</v>
@@ -3773,13 +3773,13 @@
       <c r="F36" s="8"/>
       <c r="G36" s="8"/>
       <c r="H36" s="13" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I36" s="11" t="s">
         <v>200</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
@@ -3812,7 +3812,7 @@
         <v>168</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>169</v>
@@ -3857,19 +3857,19 @@
         <v>193</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G39" s="8" t="s">
         <v>169</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="I39" s="11" t="s">
         <v>202</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>39</v>
@@ -3899,7 +3899,7 @@
         <v>146</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G40" s="8" t="s">
         <v>5</v>
@@ -3941,7 +3941,7 @@
         <v>146</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G41" s="8" t="s">
         <v>186</v>
@@ -3983,7 +3983,7 @@
         <v>146</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G42" s="8" t="s">
         <v>5</v>
@@ -4016,7 +4016,7 @@
         <v>171</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>172</v>
@@ -4025,10 +4025,10 @@
         <v>194</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H43" s="13"/>
       <c r="I43" s="11"/>
@@ -4066,7 +4066,7 @@
         <v>174</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>175</v>
@@ -4075,7 +4075,7 @@
         <v>195</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G45" s="8" t="s">
         <v>185</v>
@@ -4399,7 +4399,7 @@
         <v>198</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G54" s="8" t="s">
         <v>178</v>
@@ -4441,7 +4441,7 @@
         <v>146</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G55" s="8" t="s">
         <v>186</v>
@@ -4483,7 +4483,7 @@
         <v>146</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G56" s="8" t="s">
         <v>5</v>
@@ -4519,7 +4519,7 @@
         <v>161</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G57" s="8" t="s">
         <v>185</v>
@@ -4528,10 +4528,10 @@
         <v>161</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K57" s="2" t="s">
         <v>46</v>
@@ -4575,7 +4575,7 @@
         <v>146</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G59" s="8" t="s">
         <v>186</v>
@@ -4623,13 +4623,13 @@
         <v>185</v>
       </c>
       <c r="H60" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="I60" s="11" t="s">
         <v>202</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K60" s="2" t="s">
         <v>47</v>
@@ -4695,7 +4695,7 @@
         <v>146</v>
       </c>
       <c r="F62" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G62" s="8" t="s">
         <v>5</v>
@@ -4737,7 +4737,7 @@
         <v>146</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G63" s="8" t="s">
         <v>186</v>
@@ -4812,7 +4812,7 @@
         <v>181</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>182</v>
@@ -4821,7 +4821,7 @@
         <v>199</v>
       </c>
       <c r="F66" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G66" s="8" t="s">
         <v>182</v>
@@ -4935,7 +4935,7 @@
         <v>146</v>
       </c>
       <c r="F69" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G69" s="8" t="s">
         <v>186</v>
@@ -4996,7 +4996,7 @@
       </c>
       <c r="L70" s="2"/>
       <c r="M70" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="N70" s="2" t="s">
         <v>25</v>

</xml_diff>